<commit_message>
Use real APP test data in Store, Product and Pre-Order test cases
Replace placeholders with values from the APP: MSISDNs 504563459 /
0507127863, WHOOP PEAK BAND 5.0 (Wearables), PLUS 6TH, partnership email
test@stc.com.sa. Add a 'Real value in APP' column to Test Data with the
remaining products to fill. Raise Free Device line selection case to P1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YUiRueBr8ve5AHHG3UdcTU
</commit_message>
<xml_diff>
--- a/test-cases/MySTC_Store_Product_UI_TestCases.xlsx
+++ b/test-cases/MySTC_Store_Product_UI_TestCases.xlsx
@@ -17,8 +17,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'mystc5 Store UI Automation'!$A$1:$L$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'mystc5 Product UI Automation'!$A$1:$L$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pre-Order Coverage'!$A$1:$L$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Test Data'!$A$1:$D$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'QA Review &amp; Gaps'!$A$1:$B$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Test Data'!$A$1:$E$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'QA Review &amp; Gaps'!$A$1:$B$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -46,7 +46,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +61,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -91,6 +96,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -576,7 +584,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER</t>
+          <t>User: Public user</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -639,13 +647,13 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY</t>
+          <t>User: 504563459</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Wait until Store screen is displayed</t>
         </is>
@@ -659,7 +667,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Repeat with OTP_USER_PRIMARY</t>
+          <t>Repeat with 504563459</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -706,8 +714,8 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Categories: CAT_SMARTPHONES, CAT_WEARABLES</t>
+          <t>User: Public user
+Categories: Smart Phones, Wearables</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -720,8 +728,8 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>1- Category CAT_SMARTPHONES is displayed with its label
-2- Category CAT_WEARABLES is displayed with its label
+          <t>1- Category Smart Phones is displayed with its label
+2- Category Wearables is displayed with its label
 3- Each category label text is not empty</t>
         </is>
       </c>
@@ -770,9 +778,9 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Category: CAT_SMARTPHONES
-Expected device: DEV_NORMAL_INSTOCK (listed under Smart Phones)</t>
+          <t>User: Public user
+Category: Smart Phones
+Expected device: DEV_SMARTPHONE_INSTOCK (listed under Smart Phones)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -780,15 +788,15 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
+4- Tap category Smart Phones
 5- Observe device list</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>1- Device list for CAT_SMARTPHONES is displayed
-2- Device card DEV_NORMAL_INSTOCK is displayed in the list
-3- No Wearables-only device (DEV_WEARABLE) is displayed in the list</t>
+          <t>1- Device list for Smart Phones is displayed
+2- Device card DEV_SMARTPHONE_INSTOCK is displayed in the list
+3- No Wearables-only device (WHOOP PEAK BAND 5.0) is displayed in the list</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
@@ -836,9 +844,9 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Category: CAT_WEARABLES
-Expected device: DEV_WEARABLE</t>
+          <t>User: Public user
+Category: Wearables
+Expected device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -846,15 +854,15 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_WEARABLES
+4- Tap category Wearables
 5- Observe device list</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>1- Device list for CAT_WEARABLES is displayed
-2- Device card DEV_WEARABLE is displayed
-3- Smart-phone-only device DEV_NORMAL_INSTOCK is not displayed</t>
+          <t>1- Device list for Wearables is displayed
+2- Device card WHOOP PEAK BAND 5.0 is displayed
+3- Smart-phone-only device DEV_SMARTPHONE_INSTOCK is not displayed</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -902,8 +910,8 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Categories: CAT_SMARTPHONES, CAT_WEARABLES</t>
+          <t>User: Public user
+Categories: Smart Phones, Wearables</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -911,11 +919,11 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
+4- Tap category Smart Phones
 5- Record name of first device card as A
-6- Tap category CAT_WEARABLES
+6- Tap category Wearables
 7- Record name of first device card as B
-8- Tap category CAT_SMARTPHONES
+8- Tap category Smart Phones
 9- Record name of first device card as C</t>
         </is>
       </c>
@@ -971,8 +979,8 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Device: DEV_NORMAL_INSTOCK (known name and price)</t>
+          <t>User: Public user
+Device: WHOOP PEAK BAND 5.0 (known name and price)</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -980,13 +988,13 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Locate device card DEV_NORMAL_INSTOCK</t>
+4- Tap category Wearables
+5- Locate device card WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>1- Device name text equals DEV_NORMAL_INSTOCK name
+          <t>1- Device name text equals WHOOP PEAK BAND 5.0 name
 2- Device image is displayed (element visible, non-zero size)
 3- Price text is displayed and contains the currency and a numeric value</t>
         </is>
@@ -1036,8 +1044,8 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Device: DEV_NORMAL_INSTOCK</t>
+          <t>User: Public user
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1045,9 +1053,9 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Record name and price on device card DEV_NORMAL_INSTOCK
-6- Tap device card DEV_NORMAL_INSTOCK</t>
+4- Tap category Wearables
+5- Record name and price on device card WHOOP PEAK BAND 5.0
+6- Tap device card WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1059,7 +1067,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Repeat for logged-in user (LOGIN_USER_PRIMARY)</t>
+          <t>Repeat for logged-in user (504563459)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1106,9 +1114,9 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Category: CAT_WEARABLES
-Device: DEV_WEARABLE</t>
+          <t>User: Public user
+Category: Wearables
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1116,16 +1124,16 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_WEARABLES
-5- Tap device card DEV_WEARABLE
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Tap the Back arrow in the top-left of Device Details</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
           <t>1- Store screen is displayed
-2- CAT_WEARABLES is still the selected category
-3- Device card DEV_WEARABLE is displayed in the list</t>
+2- Wearables is still the selected category
+3- Device card WHOOP PEAK BAND 5.0 is displayed in the list</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -1177,9 +1185,9 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Category: CAT_WEARABLES
-Device: DEV_WEARABLE</t>
+          <t>User: Public user
+Category: Wearables
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1187,15 +1195,15 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_WEARABLES
-5- Tap device card DEV_WEARABLE
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Press Android system Back (driver.back())</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
           <t>1- Store screen is displayed
-2- CAT_WEARABLES is still the selected category
+2- Wearables is still the selected category
 3- APP is not closed</t>
         </is>
       </c>
@@ -1244,8 +1252,8 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Category: CAT_SMARTPHONES (contains more devices than fit on one screen)</t>
+          <t>User: Public user
+Category: Smart Phones (contains more devices than fit on one screen)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1253,7 +1261,7 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
+4- Tap category Smart Phones
 5- Record name of first device card
 6- Swipe up until no new device card appears
 7- Swipe down until the top of the list is reached</t>
@@ -1312,8 +1320,8 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Category: CAT_WEARABLES
+          <t>User: Public user
+Category: Wearables
 Device position: 6</t>
         </is>
       </c>
@@ -1322,7 +1330,7 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_WEARABLES
+4- Tap category Wearables
 5- Scroll until device card at position 6 is visible
 6- Record its name
 7- Tap it</t>
@@ -1380,14 +1388,14 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Cart: 1 x DEV_NORMAL_INSTOCK</t>
+          <t>User: 504563459
+Cart: 1 x WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Observe Cart icon</t>
         </is>
@@ -1448,14 +1456,14 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Cart: empty</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Observe Cart icon</t>
         </is>
@@ -1511,13 +1519,13 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY</t>
+          <t>User: 504563459</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Tap Cart icon</t>
         </is>
@@ -1573,18 +1581,18 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Cart: 1 x DEV_NORMAL_INSTOCK</t>
+          <t>User: 504563459
+Cart: 1 x WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap category CAT_WEARABLES
-6- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Wearables
+5- Tap category Wearables
+6- Tap category Wearables
 7- Observe Cart badge</t>
         </is>
       </c>
@@ -1639,17 +1647,17 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_NORMAL_INSTOCK</t>
+          <t>User: 504563459
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+2- Login with 504563459
+3- Tap Store
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Select purchase option Cash
 7- Tap Add to Cart
 8- Wait for Add to Cart to complete
@@ -1707,8 +1715,8 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Device: DEV_NORMAL_INSTOCK
+          <t>User: Public user
+Device: WHOOP PEAK BAND 5.0
 Taps: 5 within 1 second</t>
         </is>
       </c>
@@ -1717,8 +1725,8 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK 5 times rapidly
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0 5 times rapidly
 6- Tap Back once</t>
         </is>
       </c>
@@ -1773,7 +1781,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_DISCOUNTED (original price O, discounted price P)</t>
         </is>
       </c>
@@ -1838,7 +1846,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_NO_DISCOUNT</t>
         </is>
       </c>
@@ -1902,7 +1910,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_LONG_NAME (name &gt; 40 characters)</t>
         </is>
       </c>
@@ -1971,7 +1979,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_OOS</t>
         </is>
       </c>
@@ -1980,7 +1988,7 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
+4- Tap category Smart Phones
 5- Locate device card DEV_OOS</t>
         </is>
       </c>
@@ -2035,7 +2043,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER</t>
+          <t>User: Public user</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -2096,7 +2104,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER</t>
+          <t>User: Public user</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -2159,7 +2167,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Banners: BANNER_SET (&gt;= 2)</t>
         </is>
       </c>
@@ -2230,7 +2238,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Banner: BANNER_LINKED -&gt; target screen T</t>
         </is>
       </c>
@@ -2293,7 +2301,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Network profile: slow</t>
         </is>
       </c>
@@ -2358,7 +2366,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Network: OFF then ON</t>
         </is>
       </c>
@@ -2425,7 +2433,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Devices: smallest iOS (iPhone SE 3rd gen) and smallest Android in device matrix</t>
         </is>
       </c>
@@ -2434,7 +2442,7 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
+4- Tap category Smart Phones
 5- Observe first device card</t>
         </is>
       </c>
@@ -2494,7 +2502,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER</t>
+          <t>User: Public user</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2649,23 +2657,23 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_NORMAL_INSTOCK</t>
+          <t>User: 504563459
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+2- Login with 504563459
+3- Tap Store
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Observe Device Details screen</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>1- Device name equals DEV_NORMAL_INSTOCK name
+          <t>1- Device name equals WHOOP PEAK BAND 5.0 name
 2- Device image is displayed
 3- Price is displayed
 4- Add to Cart button is displayed and enabled
@@ -2717,16 +2725,16 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_MULTI_STORAGE</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_MULTI_STORAGE
 6- Observe color and storage selectors</t>
         </is>
@@ -2783,7 +2791,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_MULTI_STORAGE
 Storage A price PA, Storage B price PB (PA != PB)</t>
         </is>
@@ -2791,9 +2799,9 @@
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_MULTI_STORAGE
 6- Tap storage A
 7- Record price
@@ -2853,16 +2861,16 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_MULTI_COLOR (Color A, Color B, same storage)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_MULTI_COLOR
 6- Tap Color A
 7- Capture device image
@@ -2923,17 +2931,17 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_PARTIAL_OOS (Variation A out of stock, Variation B in stock)</t>
+          <t>User: 504563459
+Device: PLUS 6TH (Variation A out of stock, Variation B in stock)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_PARTIAL_OOS
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
+5- Tap device card PLUS 6TH
 6- Select Variation A
 7- Observe Add to Cart
 8- Select Variation B
@@ -2994,16 +3002,16 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_MULTI_STORAGE (A, B)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_MULTI_STORAGE
 6- Tap storage A, B, A, B, A, B (6 taps, ~300 ms apart)
 7- Observe selectors and price</t>
@@ -3061,16 +3069,16 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_ALL_OPTIONS (Cash, Installment, Free Device, Cashback)</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_ALL_OPTIONS
 6- Observe purchase options section</t>
         </is>
@@ -3130,18 +3138,18 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_NORMAL_INSTOCK
+          <t>User: 504563459
+Device: WHOOP PEAK BAND 5.0
 Purchase option: Cash</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+2- Login with 504563459
+3- Tap Store
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Select available variation
 7- Select Cash
 8- Tap Add to Cart
@@ -3158,7 +3166,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Repeat with OTP_USER_PRIMARY</t>
+          <t>Repeat with 504563459</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -3205,18 +3213,18 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_NORMAL_INSTOCK
+          <t>User: 504563459
+Device: WHOOP PEAK BAND 5.0
 Purchase option: Cash</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+2- Login with 504563459
+3- Tap Store
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Select Cash
 7- Tap Buy Now</t>
         </is>
@@ -3272,8 +3280,8 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Device: DEV_WEARABLE (normal, in stock)</t>
+          <t>User: Public user
+Device: WHOOP PEAK BAND 5.0 (normal, in stock)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -3281,8 +3289,8 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_WEARABLES
-5- Tap device card DEV_WEARABLE
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Tap Buy Now</t>
         </is>
       </c>
@@ -3337,8 +3345,8 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Device: DEV_WEARABLE</t>
+          <t>User: Public user
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -3346,8 +3354,8 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_WEARABLES
-5- Tap device card DEV_WEARABLE
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Tap Buy Now
 7- Tap Continue as a guest</t>
         </is>
@@ -3402,8 +3410,8 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Device: DEV_NORMAL_INSTOCK</t>
+          <t>User: Public user
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -3411,8 +3419,8 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Tap Add to Cart
 7- Observe screen</t>
         </is>
@@ -3468,7 +3476,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_INSTALLMENT</t>
         </is>
       </c>
@@ -3477,7 +3485,7 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
+4- Tap category Smart Phones
 5- Tap device card DEV_INSTALLMENT
 6- Select Installment
 7- Tap Buy Now</t>
@@ -3535,17 +3543,17 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_INSTALLMENT
-Line: ELIGIBLE_VOICE_POSTPAID</t>
+Line: 504563459</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_INSTALLMENT
 6- Select Installment
 7- Observe Installment section</t>
@@ -3604,21 +3612,21 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_INSTALLMENT
-Line: ELIGIBLE_VOICE_POSTPAID
+Line: 504563459
 Months: PLAN_MONTHS_1</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_INSTALLMENT
 6- Select Installment
-7- Select ELIGIBLE_VOICE_POSTPAID
+7- Select 504563459
 8- Select PLAN_MONTHS_1
 9- Tap Confirm</t>
         </is>
@@ -3679,16 +3687,16 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_INSTALLMENT</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_INSTALLMENT
 6- Select Installment
 7- Do not select number or months
@@ -3746,20 +3754,20 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_INSTALLMENT
-Line: ELIGIBLE_VOICE_POSTPAID</t>
+Line: 504563459</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_INSTALLMENT
 6- Select Installment
-7- Select ELIGIBLE_VOICE_POSTPAID
+7- Select 504563459
 8- Record amount
 9- Increase counter once
 10- Record amount
@@ -3819,16 +3827,16 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>User: OTP_USER_SECONDARY (not installment eligible)
+          <t>User: 0507127863 (not installment eligible)
 Device: DEV_INSTALLMENT</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login via OTP with OTP_USER_SECONDARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login via OTP with 0507127863
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_INSTALLMENT
 6- Select Installment</t>
         </is>
@@ -3869,7 +3877,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -3885,20 +3893,20 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_FREE_DEVICE
-Line: ELIGIBLE_VOICE_POSTPAID</t>
+          <t>User: 504563459
+Device: PLUS 6TH
+Line: 504563459</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_FREE_DEVICE
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
+5- Tap device card PLUS 6TH
 6- Select Free Device
-7- Select ELIGIBLE_VOICE_POSTPAID
+7- Select 504563459
 8- Tap Continue</t>
         </is>
       </c>
@@ -3968,7 +3976,7 @@
           <t>1- Launch MySTC APP
 2- Login with USER_NO_CASHBACK_LINE
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
+4- Tap category Smart Phones
 5- Tap device card DEV_CASHBACK
 6- Tap Cashback option</t>
         </is>
@@ -4025,7 +4033,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CASHBACK
 Line: CASHBACK_ELIGIBLE_LINE</t>
         </is>
@@ -4033,9 +4041,9 @@
       <c r="I22" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_CASHBACK
 6- Select Cashback
 7- Select CASHBACK_ELIGIBLE_LINE</t>
@@ -4093,16 +4101,16 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_DPP</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_DPP
 6- Observe DPP option
 7- Tap DPP option
@@ -4164,16 +4172,16 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_STC_PROTECT</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_STC_PROTECT
 6- Select available variation
 7- Tap Add to Cart
@@ -4235,16 +4243,16 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_STC_PROTECT</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_STC_PROTECT
 6- Select available variation
 7- Tap Add to Cart
@@ -4303,16 +4311,16 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_ONEPOOL (local stock 0, OnePool stock &gt; 0)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_ONEPOOL
 6- Observe action buttons</t>
         </is>
@@ -4372,16 +4380,16 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_ONEPOOL</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_ONEPOOL
 6- Observe delivery estimation text</t>
         </is>
@@ -4437,16 +4445,16 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_ONEPOOL_NOSTOCK (local 0, OnePool 0)</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_ONEPOOL_NOSTOCK
 6- Tap Buy Now</t>
         </is>
@@ -4504,16 +4512,16 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_ONEPOOL_NOSTOCK</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_ONEPOOL_NOSTOCK
 6- Tap Buy Now
 7- Tap Cancel</t>
@@ -4570,16 +4578,16 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_ONEPOOL_NOSTOCK</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_ONEPOOL_NOSTOCK
 6- Tap Buy Now
 7- Tap Add to wishlist</t>
@@ -4637,7 +4645,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_ONEPOOL_NOSTOCK_WEARABLE</t>
         </is>
       </c>
@@ -4646,7 +4654,7 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_WEARABLES
+4- Tap category Wearables
 5- Tap device card DEV_ONEPOOL_NOSTOCK_WEARABLE
 6- Tap Buy Now
 7- Tap Continue as a guest
@@ -4705,16 +4713,16 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_FAKE_ONEPOOL (OnePool flag but local stock &gt; 0)</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_FAKE_ONEPOOL
 6- Select Cash
 7- Observe action buttons</t>
@@ -4771,16 +4779,16 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_PREORDER_NOSTOCK</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_PREORDER_NOSTOCK
 6- Tap Notify me when available</t>
         </is>
@@ -4837,16 +4845,16 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_OOS (all variations stock 0, not pre-order)</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_OOS
 6- Observe action buttons
 7- Tap Add to Cart if displayed
@@ -4906,16 +4914,16 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_BACKORDER_RES_Y</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_BACKORDER_RES_Y
 6- Observe action buttons
 7- Tap Reserve Now
@@ -4974,16 +4982,16 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_BACKORDER_RES_N</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_BACKORDER_RES_N
 6- Observe action buttons</t>
         </is>
@@ -5040,20 +5048,20 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_PARTNERSHIP
-Email: PARTNER_EMAIL_VALID</t>
+Email: test@stc.com.sa</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_PARTNERSHIP
 6- Observe partnership email field
-7- Enter PARTNER_EMAIL_VALID
+7- Enter test@stc.com.sa
 8- Tap Add to Cart
 9- Observe Cart badge</t>
         </is>
@@ -5115,19 +5123,19 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_PARTNERSHIP
-Email: PARTNER_EMAIL_INVALID ('abc@')</t>
+Email: invalid email 'test@stc' (no domain suffix)</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_PARTNERSHIP
-6- Enter PARTNER_EMAIL_INVALID
+6- Enter invalid email 'test@stc'
 7- Tap Add to Cart
 8- Observe screen and Cart badge</t>
         </is>
@@ -5188,18 +5196,18 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_NORMAL_INSTOCK
+          <t>User: 504563459
+Device: WHOOP PEAK BAND 5.0
 Taps: 5 within 1 second</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+2- Login with 504563459
+3- Tap Store
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Select Cash
 7- Tap Add to Cart 5 times rapidly
 8- Wait until loading indicator disappears
@@ -5257,17 +5265,17 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_NORMAL_INSTOCK</t>
+          <t>User: 504563459
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+2- Login with 504563459
+3- Tap Store
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Tap Buy Now 5 times rapidly
 7- Tap Back once</t>
         </is>
@@ -5324,18 +5332,18 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Cart: PREPAID_ORDER_IN_CART
-Device: DEV_NORMAL_INSTOCK</t>
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+2- Login with 504563459
+3- Tap Store
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Record Cart badge as N
 7- Tap Add to Cart
 8- Observe screen</t>
@@ -5393,18 +5401,18 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Cart: CART_MAX_COUNT items
-Device: DEV_NORMAL_INSTOCK</t>
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+2- Login with 504563459
+3- Tap Store
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Record Cart badge as N
 7- Tap Add to Cart
 8- Observe screen</t>
@@ -5462,18 +5470,18 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_NORMAL_INSTOCK
+          <t>User: 504563459
+Device: WHOOP PEAK BAND 5.0
 Network: OFF then ON</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+2- Login with 504563459
+3- Tap Store
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Enable airplane mode
 7- Tap Add to Cart
 8- Observe screen
@@ -5535,24 +5543,24 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_NORMAL_INSTOCK</t>
+          <t>User: 504563459
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+2- Login with 504563459
+3- Tap Store
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Tap Back arrow</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
           <t>1- Store screen is displayed
-2- CAT_SMARTPHONES is still selected</t>
+2- Wearables is still selected</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
@@ -5604,24 +5612,24 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_NORMAL_INSTOCK</t>
+          <t>User: 504563459
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+2- Login with 504563459
+3- Tap Store
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Press Android system Back</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
           <t>1- Store screen is displayed
-2- CAT_SMARTPHONES is still selected</t>
+2- Wearables is still selected</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr"/>
@@ -5669,7 +5677,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_MULTI_IMAGE (&gt;= 2 images)</t>
         </is>
       </c>
@@ -5678,7 +5686,7 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
+4- Tap category Smart Phones
 5- Tap device card DEV_MULTI_IMAGE
 6- Capture image
 7- Swipe image left
@@ -5743,7 +5751,7 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_DISCOUNTED (O, P)</t>
         </is>
       </c>
@@ -5752,7 +5760,7 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
+4- Tap category Smart Phones
 5- Tap device card DEV_DISCOUNTED
 6- Observe price section</t>
         </is>
@@ -5813,8 +5821,8 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
-Device: DEV_NORMAL_INSTOCK</t>
+          <t>User: Public user
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
@@ -5822,8 +5830,8 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Scroll down to description/specifications section</t>
         </is>
       </c>
@@ -5882,17 +5890,17 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_NORMAL_INSTOCK</t>
+          <t>User: 504563459
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
-5- Tap device card DEV_NORMAL_INSTOCK
+2- Login with 504563459
+3- Tap Store
+4- Tap category Wearables
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Swipe up until end of screen
 7- Observe action buttons</t>
         </is>
@@ -5948,7 +5956,7 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_LONG_NAME</t>
         </is>
       </c>
@@ -5957,7 +5965,7 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category CAT_SMARTPHONES
+4- Tap category Smart Phones
 5- Tap device card DEV_LONG_NAME
 6- Observe device name and price</t>
         </is>
@@ -6017,16 +6025,16 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_MULTI_STORAGE</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_MULTI_STORAGE
 6- Select storage B
 7- Send APP to background for 10 seconds
@@ -6085,7 +6093,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_ALL_OPTIONS
 Screens: iPhone SE 3rd gen; smallest Android in matrix</t>
         </is>
@@ -6093,9 +6101,9 @@
       <c r="I52" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Tap category CAT_SMARTPHONES
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart Phones
 5- Tap device card DEV_ALL_OPTIONS
 6- Observe purchase options and action buttons</t>
         </is>
@@ -6246,7 +6254,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_CS_SOON_TAG_PRICE (store tag = soon, price set)</t>
         </is>
       </c>
@@ -6311,14 +6319,14 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_SOON_TAG_PRICE (store tag = soon, price set)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_SOON_TAG_PRICE</t>
         </is>
@@ -6376,14 +6384,14 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>User: OTP_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_SOON_TAG_PRICE (store tag = soon, price set)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login via OTP with OTP_USER_PRIMARY
+2- Login via OTP with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_SOON_TAG_PRICE</t>
         </is>
@@ -6441,14 +6449,14 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>User: OTP_USER_SECONDARY
+          <t>User: 0507127863
 Device: DEV_CS_SOON_TAG_PRICE (store tag = soon, price set)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login via OTP with OTP_USER_SECONDARY
+2- Login via OTP with 0507127863
 3- Tap Store
 4- Locate device card DEV_CS_SOON_TAG_PRICE</t>
         </is>
@@ -6506,16 +6514,16 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_NORMAL_INSTOCK (no soon tag)</t>
+          <t>User: 504563459
+Device: WHOOP PEAK BAND 5.0 (no soon tag)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Locate device card DEV_NORMAL_INSTOCK</t>
+2- Login with 504563459
+3- Tap Store
+4- Locate device card WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -6526,7 +6534,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Repeat for PUBLIC_USER</t>
+          <t>Repeat for Public user</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -6573,7 +6581,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_CS_SOON_TAG_NOPRICE (tag = soon, price null)</t>
         </is>
       </c>
@@ -6595,7 +6603,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Run for: PUBLIC_USER, LOGIN_USER_PRIMARY, OTP_USER_PRIMARY, OTP_USER_SECONDARY</t>
+          <t>Run for: Public user, 504563459, 504563459, 0507127863</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -6642,14 +6650,14 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_SOON_TAG_PRICE</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Record name of device card DEV_CS_SOON_TAG_PRICE
 5- Tap device card DEV_CS_SOON_TAG_PRICE</t>
@@ -6663,7 +6671,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Repeat for PUBLIC_USER</t>
+          <t>Repeat for Public user</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -6710,7 +6718,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Language: EN then AR</t>
         </is>
       </c>
@@ -6776,14 +6784,14 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_NODATE (comingSoon = Y, releaseDate null)</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_NODATE (scroll Store / category if needed)
 5- Tap device card DEV_CS_NODATE
@@ -6799,7 +6807,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Run for: PUBLIC_USER, LOGIN_USER_PRIMARY, OTP_USER_PRIMARY, OTP_USER_SECONDARY</t>
+          <t>Run for: Public user, 504563459, 504563459, 0507127863</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -6846,14 +6854,14 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_TIMER (comingSoon = Y, releaseDate = now + 2d 03h 00m)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_TIMER (scroll Store / category if needed)
 5- Tap device card DEV_CS_TIMER
@@ -6870,7 +6878,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Run for: PUBLIC_USER, LOGIN_USER_PRIMARY, OTP_USER_PRIMARY, OTP_USER_SECONDARY</t>
+          <t>Run for: Public user, 504563459, 504563459, 0507127863</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -6917,7 +6925,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_CS_TIMER</t>
         </is>
       </c>
@@ -6941,7 +6949,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Run for: PUBLIC_USER, LOGIN_USER_PRIMARY, OTP_USER_PRIMARY, OTP_USER_SECONDARY</t>
+          <t>Run for: Public user, 504563459, 504563459, 0507127863</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -6988,14 +6996,14 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_LT1DAY (releaseDate = now + 05h 00m)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_LT1DAY (scroll Store / category if needed)
 5- Tap device card DEV_CS_LT1DAY
@@ -7011,7 +7019,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Repeat for PUBLIC_USER</t>
+          <t>Repeat for Public user</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -7058,14 +7066,14 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_FAR (releaseDate = now + 120 days)</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_FAR (scroll Store / category if needed)
 5- Tap device card DEV_CS_FAR
@@ -7123,14 +7131,14 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_SHORT (comingSoon = Y, releaseDate = now + 2 min; after release the device becomes purchasable)</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_SHORT (scroll Store / category if needed)
 5- Tap device card DEV_CS_SHORT
@@ -7149,7 +7157,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Repeat for PUBLIC_USER (Buy Now becomes enabled)</t>
+          <t>Repeat for Public user (Buy Now becomes enabled)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -7196,14 +7204,14 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_TIMER</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_TIMER (scroll Store / category if needed)
 5- Tap device card DEV_CS_TIMER
@@ -7263,14 +7271,14 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_SHORT (releaseDate = now + 2 min)</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_SHORT (scroll Store / category if needed)
 5- Tap device card DEV_CS_SHORT
@@ -7331,13 +7339,13 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_TIMER</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>1- On iOS: Launch MySTC APP; Login with LOGIN_USER_PRIMARY; Tap Store; Locate device card DEV_CS_TIMER (scroll Store / category if needed); Tap device card DEV_CS_TIMER; read timer T_iOS at time X
+          <t>1- On iOS: Launch MySTC APP; Login with 504563459; Tap Store; Locate device card DEV_CS_TIMER (scroll Store / category if needed); Tap device card DEV_CS_TIMER; read timer T_iOS at time X
 2- On Android: same steps; read timer T_And at time X</t>
         </is>
       </c>
@@ -7393,7 +7401,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Devices: DEV_CS_TIMER, DEV_CS_NODATE</t>
         </is>
       </c>
@@ -7401,7 +7409,7 @@
         <is>
           <t>1- Launch MySTC APP
 2- Switch APP language to Arabic
-3- Login with LOGIN_USER_PRIMARY
+3- Login with 504563459
 4- Tap Store
 5- Tap device card DEV_CS_TIMER
 6- Observe release label and timer
@@ -7420,7 +7428,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Repeat for PUBLIC_USER</t>
+          <t>Repeat for Public user</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -7467,14 +7475,14 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_TIMER (comingSoon = Y)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_TIMER (scroll Store / category if needed)
 5- Tap device card DEV_CS_TIMER
@@ -7537,14 +7545,14 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>User: OTP_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_TIMER (comingSoon = Y)</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login via OTP with OTP_USER_PRIMARY
+2- Login via OTP with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_TIMER (scroll Store / category if needed)
 5- Tap device card DEV_CS_TIMER
@@ -7607,14 +7615,14 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>User: OTP_USER_SECONDARY
+          <t>User: 0507127863
 Device: DEV_CS_TIMER</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login via OTP with OTP_USER_SECONDARY
+2- Login via OTP with 0507127863
 3- Tap Store
 4- Locate device card DEV_CS_TIMER (scroll Store / category if needed)
 5- Tap device card DEV_CS_TIMER
@@ -7672,7 +7680,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_CS_TIMER (comingSoon = Y)</t>
         </is>
       </c>
@@ -7745,14 +7753,14 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_FLAG_NULL (comingSoon empty/null, in stock)</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_FLAG_NULL (scroll Store / category if needed)
 5- Tap device card DEV_CS_FLAG_NULL
@@ -7768,7 +7776,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Repeat for PUBLIC_USER (Buy Now enabled)</t>
+          <t>Repeat for Public user (Buy Now enabled)</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -7816,14 +7824,14 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_TIMER</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_TIMER (scroll Store / category if needed)
 5- Tap device card DEV_CS_TIMER
@@ -7884,14 +7892,14 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>User: OTP_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_TIMER</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login via OTP with OTP_USER_PRIMARY
+2- Login via OTP with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_TIMER (scroll Store / category if needed)
 5- Tap device card DEV_CS_TIMER
@@ -7951,7 +7959,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_TIMER
 Network: OFF while tapping Notify me</t>
         </is>
@@ -7959,7 +7967,7 @@
       <c r="I27" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_TIMER (scroll Store / category if needed)
 5- Tap device card DEV_CS_TIMER
@@ -8025,14 +8033,14 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_TIMER</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_TIMER (scroll Store / category if needed)
 5- Tap device card DEV_CS_TIMER
@@ -8092,14 +8100,14 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_TIMER (already in wishlist)</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_TIMER (scroll Store / category if needed)
 5- Tap device card DEV_CS_TIMER
@@ -8158,7 +8166,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_CS_NOPRICE (comingSoon = Y, price null, cashPrice null)</t>
         </is>
       </c>
@@ -8225,14 +8233,14 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_NOPRICE (comingSoon = Y, price null, cashPrice null)</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_NOPRICE (scroll Store / category if needed)
 5- Tap device card DEV_CS_NOPRICE
@@ -8249,7 +8257,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Also run for OTP_USER_PRIMARY, OTP_USER_SECONDARY</t>
+          <t>Also run for 504563459, 0507127863</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
@@ -8296,14 +8304,14 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_NOPRICE</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_NOPRICE (scroll Store / category if needed)
 5- Tap device card DEV_CS_NOPRICE
@@ -8321,7 +8329,7 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Repeat for PUBLIC_USER</t>
+          <t>Repeat for Public user</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -8368,14 +8376,14 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_TIMER (price set)</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_TIMER (scroll Store / category if needed)
 5- Tap device card DEV_CS_TIMER
@@ -8435,14 +8443,14 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_CASHONLY (comingSoon = Y, price null, cashPrice set)</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_CASHONLY (scroll Store / category if needed)
 5- Tap device card DEV_CS_CASHONLY
@@ -8501,14 +8509,14 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_PREORDER (isPreOrder = Y, releaseDate = now + 10 days)</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_PREORDER (scroll Store / category if needed)
 5- Tap device card DEV_PREORDER
@@ -8523,7 +8531,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Run for: PUBLIC_USER, LOGIN_USER_PRIMARY, OTP_USER_PRIMARY, OTP_USER_SECONDARY</t>
+          <t>Run for: Public user, 504563459, 504563459, 0507127863</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -8570,14 +8578,14 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_PREORDER_SHORT (isPreOrder = Y, releaseDate = now + 2 min)</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_PREORDER_SHORT (scroll Store / category if needed)
 5- Tap device card DEV_PREORDER_SHORT
@@ -8637,7 +8645,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_PREORDER (releaseDate = now + 61 days 12h)</t>
         </is>
       </c>
@@ -8697,14 +8705,14 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_PREORDER_NOSTOCK (isPreOrder = Y, quantity = 0)</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_PREORDER_NOSTOCK (scroll Store / category if needed)
 5- Tap device card DEV_PREORDER_NOSTOCK
@@ -8763,14 +8771,14 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>User: OTP_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_PREORDER_NOSTOCK (isPreOrder = Y, quantity = 0)</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login via OTP with OTP_USER_PRIMARY
+2- Login via OTP with 504563459
 3- Tap Store
 4- Locate device card DEV_PREORDER_NOSTOCK (scroll Store / category if needed)
 5- Tap device card DEV_PREORDER_NOSTOCK
@@ -8829,14 +8837,14 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>User: OTP_USER_SECONDARY
+          <t>User: 0507127863
 Device: DEV_PREORDER_NOSTOCK (isPreOrder = Y, quantity = 0)</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login via OTP with OTP_USER_SECONDARY
+2- Login via OTP with 0507127863
 3- Tap Store
 4- Locate device card DEV_PREORDER_NOSTOCK (scroll Store / category if needed)
 5- Tap device card DEV_PREORDER_NOSTOCK
@@ -8895,7 +8903,7 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_PREORDER_NOSTOCK (isPreOrder = Y, quantity = 0)</t>
         </is>
       </c>
@@ -8962,14 +8970,14 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_PREORDER_INSTOCK (isPreOrder = Y, quantity &gt; 0)</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_PREORDER_INSTOCK (scroll Store / category if needed)
 5- Tap device card DEV_PREORDER_INSTOCK
@@ -9030,14 +9038,14 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>User: OTP_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_PREORDER_INSTOCK (isPreOrder = Y, quantity &gt; 0)</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login via OTP with OTP_USER_PRIMARY
+2- Login via OTP with 504563459
 3- Tap Store
 4- Locate device card DEV_PREORDER_INSTOCK (scroll Store / category if needed)
 5- Tap device card DEV_PREORDER_INSTOCK
@@ -9097,7 +9105,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>User: PUBLIC_USER
+          <t>User: Public user
 Device: DEV_PREORDER_INSTOCK</t>
         </is>
       </c>
@@ -9162,14 +9170,14 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>User: OTP_USER_SECONDARY
+          <t>User: 0507127863
 Device: DEV_PREORDER_INSTOCK</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login via OTP with OTP_USER_SECONDARY
+2- Login via OTP with 0507127863
 3- Tap Store
 4- Locate device card DEV_PREORDER_INSTOCK (scroll Store / category if needed)
 5- Tap device card DEV_PREORDER_INSTOCK
@@ -9232,17 +9240,17 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
-Device: DEV_NORMAL_INSTOCK</t>
+          <t>User: 504563459
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
-3- Tap Store
-4- Locate device card DEV_NORMAL_INSTOCK (scroll Store / category if needed)
-5- Tap device card DEV_NORMAL_INSTOCK
+2- Login with 504563459
+3- Tap Store
+4- Locate device card WHOOP PEAK BAND 5.0 (scroll Store / category if needed)
+5- Tap device card WHOOP PEAK BAND 5.0
 6- Record Cart badge N
 7- Tap Add to Cart</t>
         </is>
@@ -9255,7 +9263,7 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Repeat for OTP_USER_PRIMARY</t>
+          <t>Repeat for 504563459</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
@@ -9298,19 +9306,19 @@
       <c r="G47" s="2" t="inlineStr">
         <is>
           <t>Private user - full login
-Cart contains DEV_NORMAL_INSTOCK</t>
+Cart contains WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_PREORDER_INSTOCK</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_PREORDER_INSTOCK (scroll Store / category if needed)
 5- Tap device card DEV_PREORDER_INSTOCK
@@ -9326,7 +9334,7 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>Repeat for OTP_USER_PRIMARY</t>
+          <t>Repeat for 504563459</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
@@ -9373,14 +9381,14 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>User: LOGIN_USER_PRIMARY
+          <t>User: 504563459
 Device: DEV_CS_AND_PREORDER</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
-2- Login with LOGIN_USER_PRIMARY
+2- Login with 504563459
 3- Tap Store
 4- Locate device card DEV_CS_AND_PREORDER (scroll Store / category if needed)
 5- Tap device card DEV_CS_AND_PREORDER
@@ -9412,13 +9420,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9429,15 +9438,20 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Real value in APP</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Description / required state</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Source in existing sheet</t>
         </is>
@@ -9446,973 +9460,1139 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PUBLIC_USER</t>
+          <t>LOGIN_USER_PRIMARY</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>504563459</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>User</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Not logged in; choose 'continue as public user'</t>
-        </is>
-      </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>OP4</t>
+          <t>Full login test MSISDN 504563459 (taken from existing TC sheet; test account)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>OP1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>LOGIN_USER_PRIMARY</t>
+          <t>OTP_USER_PRIMARY</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>504563459</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>User</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Full login test MSISDN 504563459 (taken from existing TC sheet; test account)</t>
-        </is>
-      </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>OP1</t>
+          <t>OTP login with primary 504563459</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>OP7</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>OTP_USER_PRIMARY</t>
+          <t>OTP_USER_SECONDARY</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>0507127863</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>User</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>OTP login with primary 504563459</t>
-        </is>
-      </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>OP7</t>
+          <t>OTP login with secondary 0507127863 - limited access</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>OP8 / OP13</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>OTP_USER_SECONDARY</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>USER_NO_CASHBACK_LINE</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>User</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>OTP login with secondary 0507127863 - limited access</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>OP8 / OP13</t>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Logged-in test user with no cashback-eligible number</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>OP21</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>USER_NO_CASHBACK_LINE</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Logged-in test user with no cashback-eligible number</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>OP21</t>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>DEV_SMARTPHONE_INSTOCK</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Normal smartphone in stock, listed only under Smart Phones (used by STORE-UI-004/005)</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>CAT_SMARTPHONES</t>
+          <t>DEV_NORMAL_INSTOCK</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Store category 'Smart Phones'</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>OP1</t>
+          <t>Normal (non-OnePool) smartphone, all variations in stock, Cash available</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Add to cart #1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CAT_WEARABLES</t>
+          <t>DEV_WEARABLE</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Store category 'Wearables'</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>Normal wearable, in stock (e.g. 6th device in Wearables)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t>OP4</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>DEV_NORMAL_INSTOCK</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>DEV_MULTI_STORAGE</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Normal (non-OnePool) smartphone, all variations in stock, Cash available</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Add to cart #1</t>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>&gt;= 2 storage variations in stock, different prices PA / PB</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Add to cart #17</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>DEV_WEARABLE</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>DEV_MULTI_COLOR</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Normal wearable, in stock (e.g. 6th device in Wearables)</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>OP4</t>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>&gt;= 2 colors in stock, same storage</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Add to cart #18</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>DEV_MULTI_STORAGE</t>
+          <t>DEV_PARTIAL_OOS</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>PLUS 6TH</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>&gt;= 2 storage variations in stock, different prices PA / PB</t>
-        </is>
-      </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Add to cart #17</t>
+          <t>Variation A stock 0, Variation B in stock</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Add to cart #19</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>DEV_MULTI_COLOR</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>DEV_OOS</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>&gt;= 2 colors in stock, same storage</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Add to cart #18</t>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Normal device, all variations stock 0, not pre-order</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Add to cart #10</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>DEV_PARTIAL_OOS</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>DEV_ALL_OPTIONS</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Variation A stock 0, Variation B in stock</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Add to cart #19</t>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Supports Cash, Installment, Free Device, Cashback</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>OP1/9/14/19</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>DEV_OOS</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>DEV_INSTALLMENT</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Normal device, all variations stock 0, not pre-order</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Add to cart #10</t>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Supports Installment</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>OP9</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>DEV_ALL_OPTIONS</t>
+          <t>DEV_FREE_DEVICE</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
+          <t>PLUS 6TH</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Supports Cash, Installment, Free Device, Cashback</t>
-        </is>
-      </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>OP1/9/14/19</t>
+          <t>Supports Free Device</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>OP14</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>DEV_INSTALLMENT</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>DEV_CASHBACK</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Supports Installment</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>OP9</t>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Supports Cashback</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>OP19</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>DEV_FREE_DEVICE</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>DEV_DPP</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Supports Free Device</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>OP14</t>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Supports DPP</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>OP2</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>DEV_CASHBACK</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>DEV_STC_PROTECT</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Supports Cashback</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>OP19</t>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Normal in-stock device eligible for STC Protect</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Add to cart #37</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>DEV_DPP</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>DEV_ONEPOOL</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Supports DPP</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>OP2</t>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>OnePool device: local stock 0, OnePool stock &gt; 0 (e.g. 3rd device in Smart Phones)</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>OP1</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>DEV_STC_PROTECT</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>DEV_ONEPOOL_NOSTOCK</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Normal in-stock device eligible for STC Protect</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Add to cart #37</t>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>OnePool device: local 0, OnePool 0</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>OP3</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>DEV_ONEPOOL</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>DEV_ONEPOOL_NOSTOCK_WEARABLE</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>OnePool device: local stock 0, OnePool stock &gt; 0 (e.g. 3rd device in Smart Phones)</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>OP1</t>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>OnePool wearable with OnePool stock 0</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>OP5</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>DEV_ONEPOOL_NOSTOCK</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>DEV_FAKE_ONEPOOL</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>OnePool device: local 0, OnePool 0</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>OP3</t>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>OnePool flag but local stock &gt; 0 (processed as normal)</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>OP25</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>DEV_ONEPOOL_NOSTOCK_WEARABLE</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>DEV_PREORDER / DEV_PREORDER_NOSTOCK</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>OnePool wearable with OnePool stock 0</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>OP5</t>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Pre-order device; NOSTOCK = stock 0 and pre-order enabled</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>OP24</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>DEV_FAKE_ONEPOOL</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>DEV_BACKORDER_RES_Y / _N</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>OnePool flag but local stock &gt; 0 (processed as normal)</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>OP25</t>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Back Order device reservable Y / N</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Add to cart #32/#40</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>DEV_PREORDER / DEV_PREORDER_NOSTOCK</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>DEV_PARTNERSHIP</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Pre-order device; NOSTOCK = stock 0 and pre-order enabled</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>OP24</t>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Device requiring partnership email</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>OP28</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>DEV_BACKORDER_RES_Y / _N</t>
+          <t>PARTNER_EMAIL_VALID / _INVALID</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
+          <t>test@stc.com.sa / test@stc</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Valid partnership email from test env / 'abc@'</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Add to cart #39</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>ELIGIBLE_VOICE_POSTPAID / ELIGIBLE_LANDLINE_POSTPAID</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>504563459 / TO FILL</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Eligible lines on LOGIN_USER_PRIMARY</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>OP9/OP10</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>CASHBACK_ELIGIBLE_LINE</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Cashback-eligible line on LOGIN_USER_PRIMARY</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>OP19</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>PLAN_MONTHS_1</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>First available installment months value</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>OP9</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>PREPAID_ORDER_IN_CART</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Cart state</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Cart contains a Prepaid Order</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Add to cart #29</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>CART_MAX_COUNT</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Cart state</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Cart filled to maximum allowed items</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Add to cart #31</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>GUEST_CONTACT</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Dummy guest contact (non-real data)</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>OP4</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>DEV_CS_TIMER</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Back Order device reservable Y / N</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Add to cart #32/#40</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>DEV_PARTNERSHIP</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>comingSoon = Y, releaseDate = now + 2d 03h 00m, price set</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>MS-2314 / MS-4095</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>DEV_CS_NODATE</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Device requiring partnership email</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>OP28</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>PARTNER_EMAIL_VALID / _INVALID</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Valid partnership email from test env / 'abc@'</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Add to cart #39</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>ELIGIBLE_VOICE_POSTPAID / ELIGIBLE_LANDLINE_POSTPAID</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Line</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Eligible lines on LOGIN_USER_PRIMARY</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>OP9/OP10</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>CASHBACK_ELIGIBLE_LINE</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Line</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Cashback-eligible line on LOGIN_USER_PRIMARY</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>OP19</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>PLAN_MONTHS_1</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>First available installment months value</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>OP9</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>PREPAID_ORDER_IN_CART</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Cart state</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Cart contains a Prepaid Order</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Add to cart #29</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>CART_MAX_COUNT</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Cart state</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Cart filled to maximum allowed items</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Add to cart #31</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>GUEST_CONTACT</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Dummy guest contact (non-real data)</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>OP4</t>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>comingSoon = Y, releaseDate empty/null, price set</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>MS-2314 P4</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>DEV_CS_TIMER</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>DEV_CS_LT1DAY / DEV_CS_FAR / DEV_CS_SHORT</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>comingSoon = Y, releaseDate = now + 2d 03h 00m, price set</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>MS-2314 / MS-4095</t>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>comingSoon = Y; releaseDate = now + 5h / + 120d / + 2 min (DEV_CS_SHORT purchasable after release)</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>MS-4095</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>DEV_CS_NODATE</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>DEV_CS_NOPRICE</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>comingSoon = Y, releaseDate empty/null, price set</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>MS-2314 P4</t>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>comingSoon = Y, price null AND cashPrice null</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>MS-2314 P8</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>DEV_CS_LT1DAY / DEV_CS_FAR / DEV_CS_SHORT</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>DEV_CS_CASHONLY</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>comingSoon = Y; releaseDate = now + 5h / + 120d / + 2 min (DEV_CS_SHORT purchasable after release)</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>MS-4095</t>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>comingSoon = Y, price null, cashPrice set</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>MS-2314 P8</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>DEV_CS_NOPRICE</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>DEV_CS_SOON_TAG_PRICE / _NOPRICE</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>comingSoon = Y, price null AND cashPrice null</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>MS-2314 P8</t>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Store tag = soon with price set / price null</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>MS-2314 P2</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>DEV_CS_CASHONLY</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>DEV_CS_FLAG_NULL</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>comingSoon = Y, price null, cashPrice set</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>MS-2314 P8</t>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>comingSoon empty/null, in stock</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>MS-2314 P3</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>DEV_CS_SOON_TAG_PRICE / _NOPRICE</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>DEV_PREORDER / DEV_PREORDER_SHORT / DEV_PREORDER_INSTOCK</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Store tag = soon with price set / price null</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>MS-2314 P2</t>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>isPreOrder = Y; releaseDate now + 10d / now + 2 min / quantity &gt; 0</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>MS-4095 P5, Add to cart #34</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>DEV_CS_FLAG_NULL</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DEV_CS_AND_PREORDER</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>comingSoon empty/null, in stock</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>MS-2314 P3</t>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>comingSoon = Y and isPreOrder = Y</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Edge</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>DEV_PREORDER / DEV_PREORDER_SHORT / DEV_PREORDER_INSTOCK</t>
+          <t>Timer setup note</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>isPreOrder = Y; releaseDate now + 10d / now + 2 min / quantity &gt; 0</t>
+          <t>Env</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>MS-4095 P5, Add to cart #34</t>
+          <t>releaseDate values are relative to test start: set them in the test environment right before the run so timer assertions stay deterministic</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>DEV_CS_AND_PREORDER</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Device</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>comingSoon = Y and isPreOrder = Y</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Timer setup note</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Env</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>releaseDate values are relative to test start: set them in the test environment right before the run so timer assertions stay deterministic</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DEV_DISCOUNTED / DEV_NO_DISCOUNT / DEV_LONG_NAME / DEV_MULTI_IMAGE / DEV_LONG_DESCRIPTION / BANNER_SET / BANNER_LINKED</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Device / Content</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>PENDING - only needed if the related UI exists</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>DEV_DISCOUNTED / DEV_NO_DISCOUNT / DEV_LONG_NAME / DEV_MULTI_IMAGE / DEV_LONG_DESCRIPTION / BANNER_SET / BANNER_LINKED</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Device / Content</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>PENDING - only needed if the related UI exists</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D45"/>
+  <autoFilter ref="A1:E43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10423,7 +10603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -10577,17 +10757,29 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>Real test data</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Values supplied by the user are written directly in the cases (504563459, 0507127863, WHOOP PEAK BAND 5.0 / Wearables, PLUS 6TH, test@stc.com.sa). Cases using WHOOP PEAK BAND 5.0 navigate via Wearables. Remaining placeholders are listed as 'TO FILL' (orange) in Test Data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>Next step</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Run the PENDING (yellow) cases against the build with Appium Inspector; delete those whose element does not exist and replace placeholders (exact texts, accessibility IDs).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B13"/>
+  <autoFilter ref="A1:B14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Align Store cases with the real Smart phones screen
Use the APP screenshot (iOS 18.4) to confirm the category screen title,
Back arrow, Cart badge, 2-column card grid, brand/name/heart/from-price,
struck-through price, out of stock and % tags, stc placeholder image and
the no internet connection banner with retry. Real products: iPhone 17
Pro Max, iPhone 15 Pro Max, Galaxy S25+, IP16PRO and AWS10 MMax 24M.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YUiRueBr8ve5AHHG3UdcTU
</commit_message>
<xml_diff>
--- a/test-cases/MySTC_Store_Product_UI_TestCases.xlsx
+++ b/test-cases/MySTC_Store_Product_UI_TestCases.xlsx
@@ -14,10 +14,10 @@
     <sheet name="QA Review &amp; Gaps" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'mystc5 Store UI Automation'!$A$1:$L$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'mystc5 Store UI Automation'!$A$1:$L$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'mystc5 Product UI Automation'!$A$1:$L$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pre-Order Coverage'!$A$1:$L$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Test Data'!$A$1:$E$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Test Data'!$A$1:$E$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'QA Review &amp; Gaps'!$A$1:$B$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -715,7 +715,7 @@
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>User: Public user
-Categories: Smart Phones, Wearables</t>
+Categories: Smart phones, Wearables</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>1- Category Smart Phones is displayed with its label
+          <t>1- Category Smart phones is displayed with its label
 2- Category Wearables is displayed with its label
 3- Each category label text is not empty</t>
         </is>
@@ -748,12 +748,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Store Screen</t>
+          <t>Store - Category Screen</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Check selecting Smart Phones category displays Smart Phones devices</t>
+          <t>Check selecting Smart phones category opens the Smart phones screen with device grid</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -779,8 +779,8 @@
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>User: Public user
-Category: Smart Phones
-Expected device: DEV_SMARTPHONE_INSTOCK (listed under Smart Phones)</t>
+Category: Smart phones
+Expected devices: iPhone 17 Pro Max, iPhone 15 Pro Max, Galaxy S25+</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -788,21 +788,24 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category Smart Phones
-5- Observe device list</t>
+4- Tap category Smart phones
+5- Observe screen</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>1- Device list for Smart Phones is displayed
-2- Device card DEV_SMARTPHONE_INSTOCK is displayed in the list
-3- No Wearables-only device (WHOOP PEAK BAND 5.0) is displayed in the list</t>
+          <t>1- Screen title 'Smart phones' is displayed
+2- Back arrow is displayed at top-left
+3- Cart icon is displayed at top-right
+4- Device cards are displayed in a 2-column grid
+5- Cards 'iPhone 17 Pro Max', 'iPhone 15 Pro Max' and 'Galaxy S25+' are displayed
+6- No Wearables device (WHOOP PEAK BAND 5.0) is displayed</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Source: existing TC sheet OP1 steps 2-3</t>
+          <t>Confirmed on APP screenshot: Smart phones category screen, iOS 18.4 simulator (iPhone 16 Pro), 4-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -862,7 +865,7 @@
         <is>
           <t>1- Device list for Wearables is displayed
 2- Device card WHOOP PEAK BAND 5.0 is displayed
-3- Smart-phone-only device DEV_SMARTPHONE_INSTOCK is not displayed</t>
+3- Smart-phone-only device iPhone 17 Pro Max is not displayed</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -873,136 +876,144 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>STORE-UI-006</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Store Screen</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Check switching category from Smart Phones to Wearables and back refreshes the device list</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>IOS &amp; Android</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>IOS &amp; Android</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Public user</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>User: Public user
-Categories: Smart Phones, Wearables</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
+Categories: Smart phones, Wearables</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Record name of first device card as A
-6- Tap category Wearables
-7- Record name of first device card as B
-8- Tap category Smart Phones
-9- Record name of first device card as C</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
+6- Tap Back arrow
+7- Tap category Wearables
+8- Record name of first device card as B
+9- Tap Back arrow
+10- Tap category Smart phones
+11- Record name of first device card as C</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>1- A is not equal to B
 2- C is equal to A
-3- Tapped category is shown in selected state each time (selected indicator moves to tapped category)</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr"/>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>Source: existing TC sheet Add to cart #25 (navigate between Store categories); selected-state indicator: PENDING UI CONFIRMATION - element/behaviour is not evidenced in the existing TC sheet. Confirm on the build (Appium Inspector) before automating; delete the case if the element does not exist.</t>
+3- Each category screen shows its own title ('Smart phones' / Wearables title)</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Source: existing TC sheet Add to cart #25; category opens its own screen with Back arrow (APP screenshot)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>STORE-UI-007</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Store Screen</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Check device card displays device name, image and price</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Store - Category Screen</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Check device card displays brand, device name, image, wishlist icon and 'from' price</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>IOS &amp; Android</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>IOS &amp; Android</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Public user</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>User: Public user
-Device: WHOOP PEAK BAND 5.0 (known name and price)</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
+Device: iPhone 17 Pro Max (brand Apple)</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category Wearables
-5- Locate device card WHOOP PEAK BAND 5.0</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>1- Device name text equals WHOOP PEAK BAND 5.0 name
-2- Device image is displayed (element visible, non-zero size)
-3- Price text is displayed and contains the currency and a numeric value</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t>Card fields inferred from Add to cart #20 (name/image/price shown for device). Exact card layout: PENDING UI CONFIRMATION - element/behaviour is not evidenced in the existing TC sheet. Confirm on the build (Appium Inspector) before automating; delete the case if the element does not exist.</t>
+4- Tap category Smart phones
+5- Locate device card 'iPhone 17 Pro Max'</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>1- Brand label 'Apple' is displayed above the device name
+2- Device name 'iPhone 17 Pro Max' is displayed
+3- Device image is displayed (visible, non-zero size)
+4- Wishlist (heart) icon is displayed on the brand label row, right side
+5- Price text matches 'from ⃁ &lt;number&gt;' (recorded: from ⃁ 5889)</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Price recorded 4-Oct-2026 - update if catalogue changes</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed on APP screenshot: Smart phones category screen, iOS 18.4 simulator (iPhone 16 Pro), 4-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1264,7 @@
       <c r="H12" s="2" t="inlineStr">
         <is>
           <t>User: Public user
-Category: Smart Phones (contains more devices than fit on one screen)</t>
+Category: Smart phones (contains more devices than fit on one screen)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1261,7 +1272,7 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Record name of first device card
 6- Swipe up until no new device card appears
 7- Swipe down until the top of the list is reached</t>
@@ -1744,325 +1755,345 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>STORE-UI-019</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Store Screen</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Check device card with discount shows original and discounted price</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Store - Category Screen</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Check device card with discount shows discounted 'from' price and struck-through original price</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>IOS &amp; Android</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>IOS &amp; Android</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Public user</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>User: Public user
-Device: DEV_DISCOUNTED (original price O, discounted price P)</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
+Device: iPhone 17 Pro Max (from ⃁ 5889, original ⃁ 9028.99)</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category of DEV_DISCOUNTED
-5- Locate device card DEV_DISCOUNTED</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>1- Discounted price P is displayed
-2- Original price O is displayed (struck-through)
-3- P is lower than O</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr"/>
-      <c r="L20" s="3" t="inlineStr">
-        <is>
-          <t>PENDING UI CONFIRMATION - element/behaviour is not evidenced in the existing TC sheet. Confirm on the build (Appium Inspector) before automating; delete the case if the element does not exist.</t>
+4- Tap category Smart phones
+5- Locate device card 'iPhone 17 Pro Max'</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>1- Discounted price 'from ⃁ 5889' is displayed
+2- Original price '⃁ 9028.99' is displayed next to it, smaller and struck-through
+3- Discounted value is lower than original value</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Prices recorded 4-Oct-2026</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed on APP screenshot: Smart phones category screen, iOS 18.4 simulator (iPhone 16 Pro), 4-Oct-2026</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>STORE-UI-020</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Store Screen</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Check device card without discount shows a single price only</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Store - Category Screen</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Check device card without discount shows a single 'from' price only</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>IOS &amp; Android</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>IOS &amp; Android</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>Public user</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>User: Public user
-Device: DEV_NO_DISCOUNT</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
+Device: iPhone 15 Pro Max (from ⃁ 2300)</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category of DEV_NO_DISCOUNT
-5- Locate device card DEV_NO_DISCOUNT</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>1- Exactly one price is displayed
-2- No struck-through price or discount label is displayed</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr"/>
-      <c r="L21" s="3" t="inlineStr">
-        <is>
-          <t>PENDING UI CONFIRMATION - element/behaviour is not evidenced in the existing TC sheet. Confirm on the build (Appium Inspector) before automating; delete the case if the element does not exist.</t>
+4- Tap category Smart phones
+5- Locate device card 'iPhone 15 Pro Max'</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>1- Price 'from ⃁ 2300' is displayed
+2- No struck-through original price is displayed
+3- No discount percentage tag is displayed</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Price recorded 4-Oct-2026</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed on APP screenshot: Smart phones category screen, iOS 18.4 simulator (iPhone 16 Pro), 4-Oct-2026</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>STORE-UI-021</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Store Screen</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Check device card with a very long device name does not overlap price or image</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Store - Category Screen</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Check device card with a long device name wraps without overlapping the price</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Edge case</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>IOS &amp; Android</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>IOS &amp; Android</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Public user</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>User: Public user
-Device: DEV_LONG_NAME (name &gt; 40 characters)</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
+Device: IP16PRO and AWS10 MMax 24M (from ⃁ 7099)</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category of DEV_LONG_NAME
-5- Locate device card DEV_LONG_NAME</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>1- Name is displayed wrapped or truncated with ellipsis
-2- Name element bounds do not intersect price element bounds
-3- Price is fully displayed</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t>Run on smallest supported device (e.g. iPhone SE, 5" Android)</t>
-        </is>
-      </c>
-      <c r="L22" s="3" t="inlineStr">
-        <is>
-          <t>PENDING UI CONFIRMATION - element/behaviour is not evidenced in the existing TC sheet. Confirm on the build (Appium Inspector) before automating; delete the case if the element does not exist.</t>
+4- Tap category Smart phones
+5- Scroll until card 'IP16PRO and AWS10 MMax 24M' is visible
+6- Observe the card</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>1- Device name is displayed on 2 lines ('IP16PRO and AWS10' / 'MMax 24M')
+2- Name bounds do not intersect price bounds
+3- Price 'from ⃁ 7099' is fully displayed below the name</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Also run on smallest supported device</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed on APP screenshot: Smart phones category screen, iOS 18.4 simulator (iPhone 16 Pro), 4-Oct-2026</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>STORE-UI-022</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Store Screen</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Check out-of-stock device is identifiable on its device card</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Store - Category Screen</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Check out-of-stock device card shows 'out of stock' tag</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Regression / Negative</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>IOS &amp; Android</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>IOS &amp; Android</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>Public user</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>User: Public user
-Device: DEV_OOS</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
+Device: Galaxy S25+ (out of stock, from ⃁ 3550)</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category Smart Phones
-5- Locate device card DEV_OOS</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>1- Device card DEV_OOS is displayed
-2- Out-of-stock / unavailable label is displayed on the card</t>
-        </is>
-      </c>
-      <c r="K23" s="3" t="inlineStr"/>
-      <c r="L23" s="3" t="inlineStr">
-        <is>
-          <t>Out-of-stock state exists (Add to cart #10); label on Store card: PENDING UI CONFIRMATION - element/behaviour is not evidenced in the existing TC sheet. Confirm on the build (Appium Inspector) before automating; delete the case if the element does not exist.</t>
+4- Tap category Smart phones
+5- Locate device card 'Galaxy S25+'</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>1- Tag with text 'out of stock' is displayed at the top-left of the card (green background)
+2- Brand 'Samsung', name 'Galaxy S25+' and price 'from ⃁ 3550' are still displayed</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Also: IP16PRO and AWS10 MMax 24M (out of stock)</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed on APP screenshot: Smart phones category screen, iOS 18.4 simulator (iPhone 16 Pro), 4-Oct-2026</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>STORE-UI-023</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Store Screen</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Check Store header title is displayed</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Store - Category Screen</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Check Back arrow on Smart phones screen returns to Store</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>IOS &amp; Android</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>IOS &amp; Android</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Public user</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>User: Public user</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Observe Store header</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>1- Header title text is displayed and equals expected Store title (EN/AR per APP language)</t>
-        </is>
-      </c>
-      <c r="K24" s="3" t="inlineStr"/>
-      <c r="L24" s="3" t="inlineStr">
-        <is>
-          <t>PENDING UI CONFIRMATION - element/behaviour is not evidenced in the existing TC sheet. Confirm on the build (Appium Inspector) before automating; delete the case if the element does not exist.</t>
+4- Tap category Smart phones
+5- Tap Back arrow at top-left</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>1- Smart phones screen is closed
+2- Store screen is displayed</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Android: also system Back</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Back arrow confirmed on APP screenshot; resulting screen per navigation</t>
         </is>
       </c>
     </row>
@@ -2328,70 +2359,74 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>STORE-UI-028</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Store Screen</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Check Store screen error state when device has no network connection</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Store - Category Screen</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Check 'no internet connection' banner is displayed on Smart phones screen when offline</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>IOS &amp; Android</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>IOS &amp; Android</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>Public user
-Device network disabled (airplane mode)</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
+Smart phones screen opened once online</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>User: Public user
 Network: OFF then ON</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>1- Launch MySTC APP
 2- Continue as public user
-3- Enable airplane mode
-4- Tap Store
-5- Observe screen
-6- Disable airplane mode
-7- Tap Retry (if displayed) or pull to refresh</t>
-        </is>
-      </c>
-      <c r="J29" s="3" t="inlineStr">
+3- Tap Store
+4- Tap category Smart phones
+5- Enable airplane mode
+6- Pull to refresh / reopen Smart phones screen
+7- Observe banner
+8- Disable airplane mode
+9- Tap retry icon in the banner</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>1- APP does not crash
-2- Error / no-connection message is displayed
-3- After network is restored and Retry is tapped, device cards are displayed</t>
-        </is>
-      </c>
-      <c r="K29" s="3" t="inlineStr"/>
-      <c r="L29" s="3" t="inlineStr">
-        <is>
-          <t>Network-failure handling: Add to cart #27 (device level). Exact Store error UI / Retry: PENDING UI CONFIRMATION - element/behaviour is not evidenced in the existing TC sheet. Confirm on the build (Appium Inspector) before automating; delete the case if the element does not exist.</t>
+2- Banner title 'no internet connection' is displayed below the screen title (red text, pink background)
+3- Banner message 'please make sure you are connected to the internet or wifi and try again' is displayed
+4- Retry (circular arrow) icon is displayed at the right of the banner
+5- After network restore and tapping retry, banner disappears and device cards are displayed</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed on APP screenshot: Smart phones category screen, iOS 18.4 simulator (iPhone 16 Pro), 4-Oct-2026 (offline state)</t>
         </is>
       </c>
     </row>
@@ -2442,7 +2477,7 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Observe first device card</t>
         </is>
       </c>
@@ -2528,8 +2563,338 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>STORE-UI-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Store - Category Screen</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Check card shows stc placeholder image when device image cannot be loaded</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Edge case</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>IOS &amp; Android</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Public user
+Device offline before images are cached</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>User: Public user
+Devices: iPhone 15 Pro Max, Galaxy S25+</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>1- Launch MySTC APP (fresh install / cleared cache)
+2- Continue as public user
+3- Tap Store
+4- Enable airplane mode
+5- Tap category Smart phones
+6- Observe card images</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>1- Cards without loaded image display the grey 'stc' placeholder image
+2- Placeholder keeps the same card size as a loaded image
+3- Brand, name and price are still displayed</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed on APP screenshot: Smart phones category screen, iOS 18.4 simulator (iPhone 16 Pro), 4-Oct-2026 (iPhone 15 Pro Max and Galaxy S25+ showed placeholder while offline)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>STORE-UI-032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Store - Category Screen</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Check discount percentage tag is displayed together with 'out of stock' tag</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>IOS &amp; Android</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Public user</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>User: Public user
+Device: DEV_DISCOUNT_PCT (out of stock + 7% discount)</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>1- Launch MySTC APP
+2- Continue as public user (do not login)
+3- Tap Store
+4- Tap category Smart phones
+5- Scroll to device card DEV_DISCOUNT_PCT</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>1- 'out of stock' tag is displayed at top-left
+2- Discount tag '7%' is displayed at top-right (orange/red)
+3- Tags do not overlap</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed on APP screenshot: Smart phones category screen, iOS 18.4 simulator (iPhone 16 Pro), 4-Oct-2026 (5th card; device name not visible on screenshot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>STORE-UI-033</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Store - Category Screen</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Check tapping wishlist heart on device card as logged-in user toggles its state</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>IOS &amp; Android</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Login
+Device not in wishlist</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>User: 504563459
+Device: iPhone 17 Pro Max</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>1- Launch MySTC APP
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart phones
+5- Tap heart icon on card 'iPhone 17 Pro Max'
+6- Observe heart
+7- Tap heart icon again
+8- Observe heart</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>1- After first tap heart is displayed filled / selected
+2- After second tap heart is displayed outlined / unselected
+3- User stays on Smart phones screen</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr"/>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>Heart icon confirmed on APP screenshot; toggle behaviour: PENDING UI CONFIRMATION - element/behaviour is not evidenced in the existing TC sheet. Confirm on the build (Appium Inspector) before automating; delete the case if the element does not exist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>STORE-UI-034</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Store - Category Screen</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Check tapping wishlist heart on device card as public user asks to login</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Regression / Negative</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>IOS &amp; Android</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Public user</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>User: Public user
+Device: iPhone 17 Pro Max</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>1- Launch MySTC APP
+2- Continue as public user (do not login)
+3- Tap Store
+4- Tap category Smart phones
+5- Tap heart icon on card 'iPhone 17 Pro Max'</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>1- Login prompt is displayed
+2- Heart stays outlined / unselected</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr"/>
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t>Heart icon confirmed on APP screenshot; public behaviour: PENDING UI CONFIRMATION - element/behaviour is not evidenced in the existing TC sheet. Confirm on the build (Appium Inspector) before automating; delete the case if the element does not exist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>STORE-UI-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Store - Category Screen</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Check Cart icon badge is displayed on Smart phones screen for user with items in Cart</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>IOS &amp; Android</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Login
+Cart contains exactly 1 item</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>User: 504563459
+Cart: 1 x WHOOP PEAK BAND 5.0</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>1- Launch MySTC APP
+2- Login with 504563459
+3- Tap Store
+4- Tap category Smart phones
+5- Observe Cart icon at top-right</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>1- Cart icon is displayed at top-right
+2- Cart badge value is 1</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed on APP screenshot: Smart phones category screen, iOS 18.4 simulator (iPhone 16 Pro), 4-Oct-2026 (badge '1')</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L31"/>
+  <autoFilter ref="A1:L36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2734,7 +3099,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_MULTI_STORAGE
 6- Observe color and storage selectors</t>
         </is>
@@ -2801,7 +3166,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_MULTI_STORAGE
 6- Tap storage A
 7- Record price
@@ -2870,7 +3235,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_MULTI_COLOR
 6- Tap Color A
 7- Capture device image
@@ -2940,7 +3305,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card PLUS 6TH
 6- Select Variation A
 7- Observe Add to Cart
@@ -3011,7 +3376,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_MULTI_STORAGE
 6- Tap storage A, B, A, B, A, B (6 taps, ~300 ms apart)
 7- Observe selectors and price</t>
@@ -3078,7 +3443,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_ALL_OPTIONS
 6- Observe purchase options section</t>
         </is>
@@ -3485,7 +3850,7 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_INSTALLMENT
 6- Select Installment
 7- Tap Buy Now</t>
@@ -3553,7 +3918,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_INSTALLMENT
 6- Select Installment
 7- Observe Installment section</t>
@@ -3623,7 +3988,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_INSTALLMENT
 6- Select Installment
 7- Select 504563459
@@ -3696,7 +4061,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_INSTALLMENT
 6- Select Installment
 7- Do not select number or months
@@ -3764,7 +4129,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_INSTALLMENT
 6- Select Installment
 7- Select 504563459
@@ -3836,7 +4201,7 @@
           <t>1- Launch MySTC APP
 2- Login via OTP with 0507127863
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_INSTALLMENT
 6- Select Installment</t>
         </is>
@@ -3903,7 +4268,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card PLUS 6TH
 6- Select Free Device
 7- Select 504563459
@@ -3976,7 +4341,7 @@
           <t>1- Launch MySTC APP
 2- Login with USER_NO_CASHBACK_LINE
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_CASHBACK
 6- Tap Cashback option</t>
         </is>
@@ -4043,7 +4408,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_CASHBACK
 6- Select Cashback
 7- Select CASHBACK_ELIGIBLE_LINE</t>
@@ -4110,7 +4475,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_DPP
 6- Observe DPP option
 7- Tap DPP option
@@ -4181,7 +4546,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_STC_PROTECT
 6- Select available variation
 7- Tap Add to Cart
@@ -4252,7 +4617,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_STC_PROTECT
 6- Select available variation
 7- Tap Add to Cart
@@ -4320,7 +4685,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_ONEPOOL
 6- Observe action buttons</t>
         </is>
@@ -4389,7 +4754,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_ONEPOOL
 6- Observe delivery estimation text</t>
         </is>
@@ -4454,7 +4819,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_ONEPOOL_NOSTOCK
 6- Tap Buy Now</t>
         </is>
@@ -4521,7 +4886,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_ONEPOOL_NOSTOCK
 6- Tap Buy Now
 7- Tap Cancel</t>
@@ -4587,7 +4952,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_ONEPOOL_NOSTOCK
 6- Tap Buy Now
 7- Tap Add to wishlist</t>
@@ -4722,7 +5087,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_FAKE_ONEPOOL
 6- Select Cash
 7- Observe action buttons</t>
@@ -4788,7 +5153,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_PREORDER_NOSTOCK
 6- Tap Notify me when available</t>
         </is>
@@ -4846,7 +5211,7 @@
       <c r="H34" s="2" t="inlineStr">
         <is>
           <t>User: 504563459
-Device: DEV_OOS (all variations stock 0, not pre-order)</t>
+Device: Galaxy S25+ (all variations stock 0, not pre-order)</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -4854,8 +5219,8 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
-5- Tap device card DEV_OOS
+4- Tap category Smart phones
+5- Tap device card Galaxy S25+
 6- Observe action buttons
 7- Tap Add to Cart if displayed
 8- Observe Cart badge</t>
@@ -4923,7 +5288,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_BACKORDER_RES_Y
 6- Observe action buttons
 7- Tap Reserve Now
@@ -4991,7 +5356,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_BACKORDER_RES_N
 6- Observe action buttons</t>
         </is>
@@ -5058,7 +5423,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_PARTNERSHIP
 6- Observe partnership email field
 7- Enter test@stc.com.sa
@@ -5133,7 +5498,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_PARTNERSHIP
 6- Enter invalid email 'test@stc'
 7- Tap Add to Cart
@@ -5686,7 +6051,7 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_MULTI_IMAGE
 6- Capture image
 7- Swipe image left
@@ -5752,7 +6117,7 @@
       <c r="H47" s="3" t="inlineStr">
         <is>
           <t>User: Public user
-Device: DEV_DISCOUNTED (O, P)</t>
+Device: iPhone 17 Pro Max (O, P)</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -5760,8 +6125,8 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category Smart Phones
-5- Tap device card DEV_DISCOUNTED
+4- Tap category Smart phones
+5- Tap device card iPhone 17 Pro Max
 6- Observe price section</t>
         </is>
       </c>
@@ -5774,7 +6139,7 @@
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Negative pair: DEV_NO_DISCOUNT shows one price only</t>
+          <t>Negative pair: iPhone 15 Pro Max shows one price only</t>
         </is>
       </c>
       <c r="L47" s="3" t="inlineStr">
@@ -5957,7 +6322,7 @@
       <c r="H50" s="3" t="inlineStr">
         <is>
           <t>User: Public user
-Device: DEV_LONG_NAME</t>
+Device: IP16PRO and AWS10 MMax 24M</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
@@ -5965,8 +6330,8 @@
           <t>1- Launch MySTC APP
 2- Continue as public user (do not login)
 3- Tap Store
-4- Tap category Smart Phones
-5- Tap device card DEV_LONG_NAME
+4- Tap category Smart phones
+5- Tap device card IP16PRO and AWS10 MMax 24M
 6- Observe device name and price</t>
         </is>
       </c>
@@ -6034,7 +6399,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_MULTI_STORAGE
 6- Select storage B
 7- Send APP to background for 10 seconds
@@ -6103,7 +6468,7 @@
           <t>1- Launch MySTC APP
 2- Login with 504563459
 3- Tap Store
-4- Tap category Smart Phones
+4- Tap category Smart phones
 5- Tap device card DEV_ALL_OPTIONS
 6- Observe purchase options and action buttons</t>
         </is>
@@ -9420,7 +9785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -9566,27 +9931,27 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>DEV_SMARTPHONE_INSTOCK</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>iPhone 17 Pro Max</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Normal smartphone in stock, listed only under Smart Phones (used by STORE-UI-004/005)</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9730,142 +10095,142 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>DEV_DISCOUNT_PCT</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Out of stock + 7% discount tag (5th card in Smart phones on 4-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>DEV_OOS</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Galaxy S25+</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Normal device, all variations stock 0, not pre-order</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Add to cart #10</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>DEV_ALL_OPTIONS</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Device</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Supports Cash, Installment, Free Device, Cashback</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>OP1/9/14/19</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>DEV_ALL_OPTIONS</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Supports Cash, Installment, Free Device, Cashback</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>OP1/9/14/19</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>DEV_INSTALLMENT</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>TO FILL</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Supports Installment</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>OP9</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>DEV_FREE_DEVICE</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>PLUS 6TH</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Supports Free Device</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>OP14</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>DEV_CASHBACK</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Device</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Supports Cashback</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>OP19</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>DEV_DPP</t>
+          <t>DEV_CASHBACK</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -9880,19 +10245,19 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Supports DPP</t>
+          <t>Supports Cashback</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>OP2</t>
+          <t>OP19</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>DEV_STC_PROTECT</t>
+          <t>DEV_DPP</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -9907,19 +10272,19 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Normal in-stock device eligible for STC Protect</t>
+          <t>Supports DPP</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Add to cart #37</t>
+          <t>OP2</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>DEV_ONEPOOL</t>
+          <t>DEV_STC_PROTECT</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -9934,19 +10299,19 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>OnePool device: local stock 0, OnePool stock &gt; 0 (e.g. 3rd device in Smart Phones)</t>
+          <t>Normal in-stock device eligible for STC Protect</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>OP1</t>
+          <t>Add to cart #37</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>DEV_ONEPOOL_NOSTOCK</t>
+          <t>DEV_ONEPOOL</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -9961,19 +10326,19 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>OnePool device: local 0, OnePool 0</t>
+          <t>OnePool device: local stock 0, OnePool stock &gt; 0 (e.g. 3rd device in Smart Phones)</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>OP3</t>
+          <t>OP1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>DEV_ONEPOOL_NOSTOCK_WEARABLE</t>
+          <t>DEV_ONEPOOL_NOSTOCK</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -9988,19 +10353,19 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>OnePool wearable with OnePool stock 0</t>
+          <t>OnePool device: local 0, OnePool 0</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>OP5</t>
+          <t>OP3</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>DEV_FAKE_ONEPOOL</t>
+          <t>DEV_ONEPOOL_NOSTOCK_WEARABLE</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -10015,19 +10380,19 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>OnePool flag but local stock &gt; 0 (processed as normal)</t>
+          <t>OnePool wearable with OnePool stock 0</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>OP25</t>
+          <t>OP5</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>DEV_PREORDER / DEV_PREORDER_NOSTOCK</t>
+          <t>DEV_FAKE_ONEPOOL</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -10042,19 +10407,19 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Pre-order device; NOSTOCK = stock 0 and pre-order enabled</t>
+          <t>OnePool flag but local stock &gt; 0 (processed as normal)</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>OP24</t>
+          <t>OP25</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>DEV_BACKORDER_RES_Y / _N</t>
+          <t>DEV_PREORDER / DEV_PREORDER_NOSTOCK</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -10069,105 +10434,105 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Back Order device reservable Y / N</t>
+          <t>Pre-order device; NOSTOCK = stock 0 and pre-order enabled</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Add to cart #32/#40</t>
+          <t>OP24</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
+          <t>DEV_BACKORDER_RES_Y / _N</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Back Order device reservable Y / N</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Add to cart #32/#40</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
           <t>DEV_PARTNERSHIP</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>TO FILL</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Device requiring partnership email</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>OP28</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>PARTNER_EMAIL_VALID / _INVALID</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>test@stc.com.sa / test@stc</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Valid partnership email from test env / 'abc@'</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Add to cart #39</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>ELIGIBLE_VOICE_POSTPAID / ELIGIBLE_LANDLINE_POSTPAID</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>504563459 / TO FILL</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Line</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>Eligible lines on LOGIN_USER_PRIMARY</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>OP9/OP10</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>CASHBACK_ELIGIBLE_LINE</t>
+          <t>ELIGIBLE_VOICE_POSTPAID / ELIGIBLE_LANDLINE_POSTPAID</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>TO FILL</t>
+          <t>504563459 / TO FILL</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -10177,19 +10542,19 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Cashback-eligible line on LOGIN_USER_PRIMARY</t>
+          <t>Eligible lines on LOGIN_USER_PRIMARY</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>OP19</t>
+          <t>OP9/OP10</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>PLAN_MONTHS_1</t>
+          <t>CASHBACK_ELIGIBLE_LINE</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -10199,24 +10564,24 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Line</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>First available installment months value</t>
+          <t>Cashback-eligible line on LOGIN_USER_PRIMARY</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>OP9</t>
+          <t>OP19</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>PREPAID_ORDER_IN_CART</t>
+          <t>PLAN_MONTHS_1</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -10226,24 +10591,24 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Cart state</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Cart contains a Prepaid Order</t>
+          <t>First available installment months value</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Add to cart #29</t>
+          <t>OP9</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>CART_MAX_COUNT</t>
+          <t>PREPAID_ORDER_IN_CART</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -10258,19 +10623,19 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Cart filled to maximum allowed items</t>
+          <t>Cart contains a Prepaid Order</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Add to cart #31</t>
+          <t>Add to cart #29</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>GUEST_CONTACT</t>
+          <t>CART_MAX_COUNT</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -10280,24 +10645,24 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Cart state</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Dummy guest contact (non-real data)</t>
+          <t>Cart filled to maximum allowed items</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>OP4</t>
+          <t>Add to cart #31</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>DEV_CS_TIMER</t>
+          <t>GUEST_CONTACT</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -10307,24 +10672,24 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>comingSoon = Y, releaseDate = now + 2d 03h 00m, price set</t>
+          <t>Dummy guest contact (non-real data)</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>MS-2314 / MS-4095</t>
+          <t>OP4</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>DEV_CS_NODATE</t>
+          <t>DEV_CS_TIMER</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -10339,19 +10704,19 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>comingSoon = Y, releaseDate empty/null, price set</t>
+          <t>comingSoon = Y, releaseDate = now + 2d 03h 00m, price set</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>MS-2314 P4</t>
+          <t>MS-2314 / MS-4095</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>DEV_CS_LT1DAY / DEV_CS_FAR / DEV_CS_SHORT</t>
+          <t>DEV_CS_NODATE</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -10366,19 +10731,19 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>comingSoon = Y; releaseDate = now + 5h / + 120d / + 2 min (DEV_CS_SHORT purchasable after release)</t>
+          <t>comingSoon = Y, releaseDate empty/null, price set</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>MS-4095</t>
+          <t>MS-2314 P4</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>DEV_CS_NOPRICE</t>
+          <t>DEV_CS_LT1DAY / DEV_CS_FAR / DEV_CS_SHORT</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -10393,19 +10758,19 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>comingSoon = Y, price null AND cashPrice null</t>
+          <t>comingSoon = Y; releaseDate = now + 5h / + 120d / + 2 min (DEV_CS_SHORT purchasable after release)</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>MS-2314 P8</t>
+          <t>MS-4095</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>DEV_CS_CASHONLY</t>
+          <t>DEV_CS_NOPRICE</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -10420,7 +10785,7 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>comingSoon = Y, price null, cashPrice set</t>
+          <t>comingSoon = Y, price null AND cashPrice null</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -10432,7 +10797,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>DEV_CS_SOON_TAG_PRICE / _NOPRICE</t>
+          <t>DEV_CS_CASHONLY</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -10447,19 +10812,19 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Store tag = soon with price set / price null</t>
+          <t>comingSoon = Y, price null, cashPrice set</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>MS-2314 P2</t>
+          <t>MS-2314 P8</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>DEV_CS_FLAG_NULL</t>
+          <t>DEV_CS_SOON_TAG_PRICE / _NOPRICE</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -10474,19 +10839,19 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>comingSoon empty/null, in stock</t>
+          <t>Store tag = soon with price set / price null</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>MS-2314 P3</t>
+          <t>MS-2314 P2</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>DEV_PREORDER / DEV_PREORDER_SHORT / DEV_PREORDER_INSTOCK</t>
+          <t>DEV_CS_FLAG_NULL</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -10501,98 +10866,125 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>isPreOrder = Y; releaseDate now + 10d / now + 2 min / quantity &gt; 0</t>
+          <t>comingSoon empty/null, in stock</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>MS-4095 P5, Add to cart #34</t>
+          <t>MS-2314 P3</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
+          <t>DEV_PREORDER / DEV_PREORDER_SHORT / DEV_PREORDER_INSTOCK</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>isPreOrder = Y; releaseDate now + 10d / now + 2 min / quantity &gt; 0</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>MS-4095 P5, Add to cart #34</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
           <t>DEV_CS_AND_PREORDER</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>TO FILL</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>comingSoon = Y and isPreOrder = Y</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E42" s="4" t="inlineStr">
         <is>
           <t>Edge</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Timer setup note</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Env</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>releaseDate values are relative to test start: set them in the test environment right before the run so timer assertions stay deterministic</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>DEV_DISCOUNTED / DEV_NO_DISCOUNT / DEV_LONG_NAME / DEV_MULTI_IMAGE / DEV_LONG_DESCRIPTION / BANNER_SET / BANNER_LINKED</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>iPhone 17 Pro Max / iPhone 15 Pro Max / IP16PRO and AWS10 MMax 24M / TO FILL / TO FILL / TO FILL / TO FILL</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>Device / Content</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>PENDING - only needed if the related UI exists</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E43"/>
+  <autoFilter ref="A1:E44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10654,7 +11046,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Store: 30 cases (15 pending). Product: 51 cases (17 pending).</t>
+          <t>Store: 35 cases (9 pending). Product: 51 cases (17 pending).</t>
         </is>
       </c>
     </row>
@@ -10738,7 +11130,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Store: header title, Search, banners &amp; indicators, banner links, loading skeleton, error/Retry UI, empty category, discount/badge labels on cards, horizontal category overflow, Wishlist icon on Store. Product: image gallery &amp; zoom, Share icon, header Wishlist/Cart icons, discount display, description/specifications, sticky action bar, quantity +/- control (not referenced in existing sheet), Notify-me confirmation, invalid email error text, Arabic/RTL layout, device rotation. Existing 'Pre-Order Coverage' sheet is empty (only a stray 's' in T13).</t>
+          <t>Confirmed from APP screenshot (Smart phones screen): title, Back arrow, Cart icon + badge, 2-column grid, brand/name/heart/from-price, struck-through price, out of stock tag, % tag, stc placeholder image, no-internet banner + retry. Still not observed - Store: Store home layout, Search, banners &amp; indicators, loading skeleton, empty category. Product: image gallery &amp; zoom, Share icon, header Wishlist/Cart icons, discount display, description/specifications, sticky action bar, quantity +/- control (not referenced in existing sheet), Notify-me confirmation, invalid email error text, Arabic/RTL layout, device rotation. Existing 'Pre-Order Coverage' sheet is empty (only a stray 's' in T13).</t>
         </is>
       </c>
     </row>

</xml_diff>